<commit_message>
Fix broken logo and null countries in fintech data
- Replace external SVG logo with styled text header
- Fix 7 fintech companies with missing country data
- Fix bad company names (Yoco, Zeepay, PalmPay, Amole)
</commit_message>
<xml_diff>
--- a/fintech_africa_leads.xlsx
+++ b/fintech_africa_leads.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Companies" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 10" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,13 +33,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -49,22 +43,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B5E20"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFECB3"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,25 +66,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -474,23 +439,23 @@
   <dimension ref="A1:Q37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="35" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -581,1857 +546,1841 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Flutterwave</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>in San Francisco, and Nigeria, and local offices everywhere in between</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>https://flutterwave.com</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>media@flutterwave.com</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Endless possibilities for every business - Flutterwave Endless possibilities for all Empowering businesses of all sizes with seamless payment solutions tailored for enterprises, startups, and emerging markets. Contact sales SweetPOD E25 Dresses Send money home to loved ones, sell online as a small business, process global payments as an enterprise, build financial products as a startup. We are trusted by leading businesses across different sectors Endless payment possibilities for enterprises Online Checkout Our online checkout features our smart payment ordering system, incredible speed, a...</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>payments, mobile money, POS, credit, cross-border, remittance, FX, API, insurance, DeFi</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Unicorn</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Diverse product offering; Late-stage / major funding; Pan-African presence (10 markets); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Major partnerships</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>EMI, SEC</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>https://flutterwave.com</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Moniepoint Inc.</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t xml:space="preserve">2026 How customer feedback drives product strategy at Moniepoint by Iwalola Sobowale Get more stories like this Sign up </t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>https://moniepoint.com</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
         <is>
           <t>0201 888 9990</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Powering Financial Dreams In Emerging Markets | Moniepoint Inc Select Region/Country Global Nigeria Kenya You are on our Global Page. Global Africa's fastest growing financial institution 2023-2025 Financial happiness for every African, everywhere Moniepoint provides an all-in-one payments, banking and operations platform for businesses and their customers. Simple financial solutions for businesses and their customers. Focus areas: payments, digital payments, digital wallet, POS, lending. Regulatory: Central Bank, EMI, microfinance bank, MFB.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>payments, digital payments, digital wallet, POS, lending, credit, loans, microfinance, digital bank, cross-border</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Listed, Unicorn, Investment, Funding, Investors</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; Late-stage / major funding; B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Central Bank, EMI, microfinance bank, MFB, SEC</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>https://moniepoint.com</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>FairMoney</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Plot 642C Akin Adesola St</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>https://www.getcarbon.co</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
         <is>
           <t>02013301808</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Personal Business Sign Up Create free account We are a bank and our superpower is giving you access to credit Instant loans, Savings, and more. Get Carbon CBN Licensed NDIC Licensed Stay in control of your money with a Carbon account Digital Esusu/Ajo Free credit report Monthly interest payout on your account Open a Carbon account Instant Loans We make access to loans simple and easy. Make online or offline payments with ease, get instant payment notifications, manage card security in app and also enjoy the benefits of spreading payments and earning monthly cashback. Focus areas: payments, ...</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>payments, POS, lending, credit, loans, microfinance, API, insurance, savings, investment</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Investment</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; Growth-stage funding; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence; Contact info available</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>CBN licensed, CBN, Central Bank, licensed, regulated, EMI, microfinance bank, SEC</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>https://www.getcarbon.co</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Mono</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Company Name Industry Select your industry Technology Finance Healthcare Educati</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>https://mono.co</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>sales@mono.co</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>652405268</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Powering African businesses with Open Banking Products Products Get high-quality customer data and build better experiences with the right APIs. See a Demo Financial Data Connect Get real-time financial data Statement Pages No-code bank statements Data Enrichment Get enriched granular insights Creditworthiness Verify credit eligibility Payments DirectPay One-time bank payments DirectDebit Recurring bank payments Global Standing Mandate Global Standing Orders Identity verification Lookup Verify government-issued IDs Prove Verify customer identity Use cases Use cases Get high-quality customer...</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>payments, POS, lending, credit, loans, microfinance, open banking, API, insurance, savings</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Investment, Raised, Funding, Investors, Backed By</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>EMI, microfinance bank, FCA, SEC</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>https://mono.co</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Kora (KoraHQ)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Thanks for subscribing! Oops! Something went wrong while submitting the form</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>https://www.korahq.com</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>support@korapay.com</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>+234 700 567 2729</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Kora | Pan-African payment infrastructure NG Log in Sign up Contact Sales Download the Startup Launch Bundle: Everything you need to build from zero and scale. The new standard for payments across Africa Simplified payments settlements collections for your business The new standard for payments across Africa Get Started Contact Sales Trusted by thousands of local and global premium brands. Build the best payment experience for Your Customers All supported by a dedicated team providing you all the support you need. Focus areas: payments, mobile money, mobile wallet, POS, credit. Regulatory: ...</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>payments, mobile money, mobile wallet, POS, credit, loans, cross-border, payment gateway, open banking, API</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Funding, Investment</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; Growth-stage funding; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Major partnerships</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>PCI, EMI, ISO 27001, SEC</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>https://www.korahq.com</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Stitch</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>3 payment gateways at the same time and Stitch Express was the quickest and easiest, so I use them</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>https://stitch.money</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>info@stitch.money</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
         <is>
           <t>Stitch Money | Online payments South Africa | Payment gateway and API Contact Sales Contact Sales Enterprise Express Enterprise payments. South Africa’s most reliable payment gateway. An end-to-end payments platform designed to optimise payments performance and streamline financial operations. Focus areas: payments, POS, point of sale, credit, payment gateway. Regulatory: PCI DSS, PCI, PSP, EMI.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>payments, POS, point of sale, credit, payment gateway, open banking, API, investment, BNPL, buy now pay later</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Investment, Raised, Funding, Investors, Backed By</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>PCI DSS, PCI, PSP, EMI, ISO 27001, SEC</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>https://stitch.money</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Peach Payments</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
         <is>
           <t>https://www.peachpayments.com</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>support@peachpayments.com</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>668342244</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Peach Payments | The Payment Orchestration Experts Orchestrating Payments For Africa's Most Exciting Enterprise Businesses Skip to content Home Page V9 (slider No Lenis) Hero Slide 1 Orchestrated Payments. Orchestrate seamless online and in-store payments to maximise conversions and drive growth. Think bigger with advanced orchestration, enterprise-grade security, alternative payment methods, and 365-day support. Focus areas: payments, digital wallet, POS, point of sale, credit. Regulatory: PCI DSS, PCI, EMI, SEC.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>payments, digital wallet, POS, point of sale, credit, payment gateway, API, BNPL</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Major partnerships</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>PCI DSS, PCI, EMI, SEC</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>https://www.peachpayments.com</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Ozow</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>to a merchant, the related billing, and service activation are subject to the re</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>https://www.ozow.com</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>sales@ozow.com</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>Secure Pay by Bank | Online Payment Gateway &amp; Bank API  | Ozow Read about our Vegas giveaway Accept payments, issue refunds &amp; make payouts, easily &amp; fast. Ozow links businesses of all sizes in South Africa with 47 million bank account holders to transact simply and securely. Become a Merchant Contact sales Download our E-commerce Report Accept payments, issue refunds &amp; make payouts, easily and fast. Focus areas: payments, POS, credit, payment gateway, open banking. Regulatory: licensed, PCI DSS, PCI, GDPR.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>payments, POS, credit, payment gateway, open banking, API, fraud detection</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Backed By</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence; Contact info available; Major partnerships</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>licensed, PCI DSS, PCI, GDPR, SEC</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q9" s="2" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>https://www.ozow.com</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Weaverfintech</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>providing financial advisory and management services to the family and their pri</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>https://www.weaverfintech.com</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
         <is>
           <t>+230 249 6740</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Home - Weaverfintech View our latest results: View Annual results View Analyst presentation Webcast What we do Fintech Our ecosystem Lending Payments Insurance Merchants Retail Who we do it for Our customer Our people Financial inclusion Development trust Our company Our structure Our board and team Results SENS Our news Contact → Where innovation meets inclusion We’re building a world where her financial journey is simple, confident, and always connected. From lending to lifestyle, we empower over 4 million South Africans to shop, lend, insure and thrive – on her terms, in her time. Our ec...</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>payments, POS, lending, credit, API, insurance, investment, BNPL</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Funding, Investment</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Professional web presence; Major partnerships</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>regulated, EMI, SEC</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q10" s="2" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>https://www.weaverfintech.com</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Adumo</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>* Phone Number * Retail Industry / Sector * Contact adumo | Your expert partner</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>https://www.adumo.com</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>sales@adumoonline.com</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>086 111 1665</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Multi-Channel Payment Solutions &amp; Card Machines | adumo ✖ 086 111 1665 sales@adumo. com Refer &amp; Earn Log in Refer &amp; earn Card machines Payments Online Capital Gift &amp; Loyalty Payouts Africa Partners POS Contact Your expert partner in payments. Whether you're a growing business or steering a large-scale enterprise, we're committed to streamlining your payment process in-store and online. Focus areas: payments, POS, lending, credit, payment gateway. Regulatory: EMI, SEC.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>payments, POS, lending, credit, payment gateway, API, insurance, BNPL, buy now pay later, identity</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Funding</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence; Contact info available; Major partnerships</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>EMI, SEC</t>
         </is>
       </c>
-      <c r="O11" s="2" t="n">
+      <c r="O11" t="n">
         <v>2021</v>
       </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q11" s="2" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>https://www.adumo.com</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>TymeBank</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>South Africa</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>of the Long-term Insurance Ombud (OLTI); and the Short-Term Insurance Ombudsman</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>https://www.tymebank.co.za</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
         <is>
           <t>0860 999 119</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Free Bank Accounts - Personal &amp; Business Banking | TymeBank Skip to content TymeBank is now GoTyme Bank. Buy your online vouchers on the TymeBank App. PayShap makes payments simple, FREE and instant just for you. Focus areas: payments, POS, point of sale, credit, digital bank. Regulatory: SEC.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>payments, POS, point of sale, credit, digital bank, payment gateway, API, insurance, savings, identity</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Funding, Backed By</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Major partnerships</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q12" s="2" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>https://www.tymebank.co.za</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>M-KOPA</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Kenya</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>27 Old Gloucester Street Bloomsbury, London, United Kingdom WC1N 3AX Supplier T&amp;</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>https://m-kopa.com</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>info@m-kopa.com</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>+254 707 333 222</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>For payments to M-KOPA Kenya use our official MPESA Pay Bill Number - 333222. For support, call +254 707 333 222 Global It seems you're viewing from Ghana Kenya South Africa Nigeria Uganda Dismiss Go to country page Get More Than a Phone Unlocking Progress for Everyday earners through easy ownership. Get your smartphone Trusted by over ‍ 7 million customers across five markets Smart Phone Unlocking financial progress with M-KOPA smart devices Value Added Services Do More. Focus areas: payments, POS, lending, credit, loans. Regulatory: EMI, SEC.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>payments, POS, lending, credit, loans, API, insurance, savings, investment, DeFi</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Investment, Investors, Backed By, Series A</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; Pan-African presence (13 markets); B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence; Contact info available; Established 15+ years</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>EMI, SEC</t>
         </is>
       </c>
-      <c r="O13" s="2" t="n">
+      <c r="O13" t="n">
         <v>2010</v>
       </c>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q13" s="2" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>https://m-kopa.com</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Tala</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Kenya</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>locations offer space for us to collaborate and connect in person — from Nairobi</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>https://tala.co</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>press@tala.co</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>Tala | Digital Financial Services, Credit, Savings and More Skip to content Powerful financial infrastructure for the new global economy Rooted in data and driven by vision, Tala is making financial services smarter, faster, and more accessible worldwide. Learn why Learn why The most comprehensive AI credit engine Tala’s personalized credit platform harnesses machine learning models trained on billions of proprietary data points from over a decade of customer relationships to underwrite millions of customers who have never interacted with the formal banking system. Data-obsessed , verticall...</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>payments, digital wallet, POS, lending, credit, loans, API, savings, investment, crypto</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Investment, Investors</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence; Contact info available; Established 11+ years; Major partnerships</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="O14" s="2" t="n">
+      <c r="O14" t="n">
         <v>2014</v>
       </c>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q14" s="2" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>https://tala.co</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Sevi</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Kenya</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
         <is>
           <t>https://www.sevi.io</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>support@sevi.io</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>254111534438</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Grow your wholesale or retail business with low-interest credit and state-of-the-art technology. Whether you’re a buyer who lacks the cash on hand to make key purchases or a seller who wants to push more products, credit unlocks new ways to grow. Leveraging state-of-the-art technology and AI, Sevi makes it easy to buy or sell on credit and track your performance along. Focus areas: payments, POS, credit, API, KYC. Regulatory: Central Bank, licensed.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>payments, POS, credit, API, KYC</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Central Bank, licensed</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="2" t="inlineStr">
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q15" s="2" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>https://www.sevi.io</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Chipper Cash</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>I made dollar payments without having to physically scout for dollars</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>https://chippercash.com</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>Save Preference Reject X Move Your Money Freely Your free Chipper account unlocks international transfers, payment cards and investing for Africans. Download the app Scan to download App Store Google Play Chipper Cash key figures 5,000,000+ Users 1,000,000+ Virtual Visa Chipper Cards Issued 6,000+ US public companies to invest in 250,000+ Transactions Per Day African payment infrastructure with global ambitions Discover Chipper for Business Send Money Directly to Bank and Mobile Money Accounts in 21+ African Countries Sending money back home just got a whole lot easier with Chipper. 4 out o...</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>payments, mobile money, POS, cross-border, investment</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>Investment</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; Pan-African presence (6 markets); B2B/infrastructure play (Payment Platform); Scale indicators (millions); Major partnerships</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="O16" s="2" t="n">
+      <c r="O16" t="n">
         <v>2020</v>
       </c>
-      <c r="P16" s="2" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q16" s="2" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>https://chippercash.com</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>expressPay</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
         <is>
           <t>https://www.expresspaygh.com</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>info@expresspaygh.com</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>+233 30 700 0503</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>expressPay The way to go Send money and make purchases with approved merchants. Give your customers a priceless payment experience when they pay for goods and services. Our API integration works across multiple platforms and also accepts both card and mobile money payments. Focus areas: payments, mobile money, POS, point of sale, remittance. Regulatory: PCI DSS, PCI, EMI, SEC.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>payments, mobile money, POS, point of sale, remittance, payment gateway, API, insurance, investment</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Investment</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Established 13+ years; Major partnerships</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>PCI DSS, PCI, EMI, SEC</t>
         </is>
       </c>
-      <c r="O17" s="2" t="n">
+      <c r="O17" t="n">
         <v>2012</v>
       </c>
-      <c r="P17" s="2" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q17" s="2" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>https://www.expresspaygh.com</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Selcom</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Tanzania</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>0800 714 888 Bofya hapa kufika SXC Manzese Morogoro Road</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>https://www.selcom.net</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>info@selcom.net</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>0800 714 888</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Selcom 0 Selcom Pesa Bridging Gaps and Driving Economic Depth Get Selcom Pesa Selcom is a Pan African cross-segment financial and payment services provider. By integrating banks, agents, and merchants into a unified ecosystem, we provide the essential infrastructure for digital, card, and card-less processing. Our turn-key solutions, which include mobile banking, e-commerce, and regional remittance corridors, empower government institutions and global enterprises alike. Focus areas: payments, digital payments, mobile money, mobile wallet, POS. Regulatory: regulated, payment service provider...</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>payments, digital payments, mobile money, mobile wallet, POS, microfinance, cross-border, remittance, API, insurance</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Ipo</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>Diverse product offering; Late-stage / major funding; B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Established 24+ years; Major partnerships</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>regulated, payment service provider, EMI, microfinance bank, SEC</t>
         </is>
       </c>
-      <c r="O18" s="2" t="n">
+      <c r="O18" t="n">
         <v>2001</v>
       </c>
-      <c r="P18" s="2" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q18" s="2" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>https://www.selcom.net</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>onafriq</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>51 Eastcheap, London, EC3M 1JP, United Kingdom Africa's Largest Digital Payments</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>https://www.beyonic.com</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>Africa's Largest Digital Payments Gateway | Onafriq The access you need to scale your business Connect your business to a real-time payments network built for Africa and get access to 1 billion wallets across the continent. Contact Sales 1B connected mobile wallets At Onafriq, the only currency that matters is access. We believe that making a payment should be as simple as a phone call. Focus areas: payments, digital payments, mobile money, mobile wallet, digital wallet. Regulatory: CBN, licensed, payment service provider, SEC.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>payments, digital payments, mobile money, mobile wallet, digital wallet, digital bank, cross-border, agent banking, agent network</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>Digital Bank / Neobank</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; Pan-African presence (11 markets); Scale indicators (millions); Major partnerships</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>CBN, licensed, payment service provider, SEC</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr"/>
-      <c r="P19" s="2" t="inlineStr">
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q19" s="2" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>https://www.beyonic.com</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Xente - Modern Payment Solutions for Africa</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Phone Number Which solutions interest you? (Select all that apply) Collect Payme</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>https://www.xente.co</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>business@xente.co</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>1478 2255 4595</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Xente - Modern Payment Solutions for Africa Payment solutions built for businesses Accept payments, send money, and access financial services seamlessly. One platform for all your payment needs across Africa. Collect local payments from anywhere in the world Make local payments across Africa instantly Access favourable treasury and liquidity for settlements Get Started Free Schedule a Demo Total Revenue 45,890,000 +12. Focus areas: payments, mobile money, mobile wallet, POS, cross-border. Regulatory: EMI, SEC.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>payments, mobile money, mobile wallet, POS, cross-border, remittance, FX, API, KYC, payroll</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>Diverse product offering; Pan-African presence (14 markets); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Major partnerships</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>EMI, SEC</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
-      <c r="P20" s="2" t="inlineStr">
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q20" s="2" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>https://www.xente.co</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Pesapal</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Kenya</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>systems for increased data validity 5</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>https://www.pesapal.com</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
         <is>
           <t>Financial Services That Drive Growth - Kenya | Pesapal Welcome to Pesapal Start Accepting M-Pesa and Card Payments Give your customers the flexibility and convenience they need by accepting both M-Pesa and card payments on one Point of sale machine. Streamline M-Pesa Till, Paybill and Xpress payments Issue M-Pesa Payment Receipts Control M-Pesa Collections Process VISA and MasterCard payments Access credit for your business Get Started Find the Solution that Fits Your Business Simplify operations, boost efficiency, and enhance customer experience with solutions tailored to fit your needs. P...</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>payments, digital payments, mobile money, POS, point of sale, lending, credit, loans, payment gateway, API</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
         <is>
           <t>Diverse product offering; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence; Major partnerships</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>payment service provider, EMI, SEC</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr"/>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q21" s="2" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>https://www.pesapal.com</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Fido - Quick Loans | Affordable Personal &amp; Business Loans in Ghana</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>to access instant loans in Ghana with Fido</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>https://www.fido.money</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>info@fido.money</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>+233 596 922 420</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Get credit, save money, and handle bills 24/7. See why millions of Africans love Fido How Fido works. At Fido, we're dedicated to offering clear, fast, and customer-focused lending. Focus areas: mobile money, POS, lending, credit, loans. Regulatory: SEC.</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>mobile money, POS, lending, credit, loans, DeFi, identity</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
         <is>
           <t>Diverse product offering; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr"/>
-      <c r="P22" s="2" t="inlineStr">
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q22" s="2" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>https://www.fido.money</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>OPay ｜ We are Beyond Banking</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>HQ: Alexander House, Plot 9, Dr</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>https://opayweb.com</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>whistleblower01@opay-inc.com</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>0700 8888 328</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>OPay ｜ We are Beyond Banking We are Beyond Banking We are Beyond Banking OPay offers secure, easy, and affordable financial solutions. Enjoy fast transactions, incentives,
             and a reliable debit card. Simplify your finances and payments, all on one efficient platform. Focus areas: payments, POS, microfinance, crypto, fraud detection. Regulatory: PCI DSS, PCI, microfinance bank, SEC.</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>payments, POS, microfinance, crypto, fraud detection, agent network</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L23" s="3" t="inlineStr">
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; B2B/infrastructure play (Payment Platform); Professional web presence</t>
         </is>
       </c>
-      <c r="N23" s="3" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>PCI DSS, PCI, microfinance bank, SEC</t>
         </is>
       </c>
-      <c r="O23" s="3" t="inlineStr"/>
-      <c r="P23" s="3" t="inlineStr">
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q23" s="3" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>https://opayweb.com</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Interswitch</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr"/>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
         <is>
           <t>https://www.interswitchgroup.com</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
         <is>
           <t>Interswitch | Powering Digital Payments Across Africa solutions products company resources Back Financial Services Driving secure and seamless transactions Wellness Digitizing care for better outcomes Energy Powering efficiency across the energy value chain Real Estate Smart living solutions for renting &amp; owning properties Mobility Shaping smarter, Safer journeys Government Innovative, efficient solutions for public service Back Individual Seamless tools to simplify everyday life Small businesses Smart payment &amp; growth enablers for SMEs Enterprise Robust platforms for organisations Develope...</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>payments, digital payments, POS, remittance, API, identity, agent network</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr"/>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>Regulated / licensed; Diverse product offering; B2B/infrastructure play (Payment Platform); Professional web presence; Established 23+ years</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>Central Bank, EMI, SEC</t>
         </is>
       </c>
-      <c r="O24" s="3" t="n">
+      <c r="O24" t="n">
         <v>2002</v>
       </c>
-      <c r="P24" s="3" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q24" s="3" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>https://www.interswitchgroup.com</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Lami Website | Homepage</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Kenya</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
         <is>
           <t>https://www.lami.world</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>antonina@lami.world</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
         <is>
           <t>Lami Website | Homepage Enabling Insurance agents to seamlessly manage their insurance
                 process. Lami is an end-to-end digital insurance platform enabling
@@ -2440,1227 +2389,845 @@
                 customers in one integrated platform. Focus areas: payments, POS, API, insurance, investment.</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>payments, POS, API, insurance, investment, agent network</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Investment, Investors, Backed By</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="L25" s="3" t="inlineStr">
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Professional web presence</t>
         </is>
       </c>
-      <c r="N25" s="3" t="inlineStr"/>
-      <c r="O25" s="3" t="inlineStr"/>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q25" s="3" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>https://www.lami.world</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Yoco | POS Systems &amp; Card Machines for Small Businesses</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr"/>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Yoco</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>1 option below Neo Touch Khumo Khumo Print Gateway Point of sale Link Invoices Xero integration Not sure about the produ</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>https://www.yoco.com</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr"/>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
         <is>
           <t>Yoco | POS Systems &amp; Card Machines for Small Businesses Login Support Get started 202,107 businesses run smarter with Yoco Save time, money and guesswork Market leader in card machines, online payments, point of sale solutions and flexible business funding, all in one place. Card machines Never miss a sale, anywhere Point of sale One system to sell, track, manage Reporting &amp; insights Know your numbers in real time Online payments Turn browsers into buyers, easily HOW YOCO CAN HELP YOUR BUSINESS Smart, reliable point of sale systems and card machines. Yoco Counter All-in-one POS and payments...</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>payments, POS, point of sale</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>Funding</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>Growth-stage funding; B2B/infrastructure play (Payment Platform)</t>
         </is>
       </c>
-      <c r="N26" s="3" t="inlineStr"/>
-      <c r="O26" s="3" t="inlineStr"/>
-      <c r="P26" s="3" t="inlineStr">
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
         <is>
           <t>בינונית</t>
         </is>
       </c>
-      <c r="Q26" s="3" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>https://www.yoco.com</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Wave</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Senegal</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Manager Abidjan, Côte d'Ivoire Office Manager Banjul, The Gambia People Operatio</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>https://www.wave.com</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
         <is>
           <t>Wave Mobile money, reinvented Deposit, withdraw, pay bills for free. Firmin Wave Build the future of money, Africa-first Join our global team bringing modern, affordable banking services to those who need them the most. Open Roles All departments Agent Operations Engineering Executive Operations and General Management Finance Growth Distribution and Sales Legal Marketing People Operations Product Risk &amp; Fraud Support All offices Burkina Faso (BF) Cameroon (CM) Cote d'Ivoire (CI) Democratic Republic of the Congo (CD) Gambia (GM) Launch Mali (ML) Niger (NE) OpCo Remote Senegal (SN) Sierra Leo...</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>payments, mobile money, POS, remittance, API</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>Investors, Backed By</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="L27" s="3" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>Diverse product offering; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence</t>
         </is>
       </c>
-      <c r="N27" s="3" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>EMI, SEC</t>
         </is>
       </c>
-      <c r="O27" s="3" t="inlineStr"/>
-      <c r="P27" s="3" t="inlineStr">
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q27" s="3" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>https://www.wave.com</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Spaceship</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr"/>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Zeepay</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>is not valid Phone Number * 000 Select country Close After entering your persona</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>https://www.zeepay.com</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>The playful combination of "zee" and "pay" hints at speed, efficiency, and modernity, making it perfect for startups in the financial technology or payment processing industries. Free transaction support Secure payments Spaceship reliability Listed with spaceship. Payment methods Submit your offer You will be redirected to spaceship. Focus areas: payments, identity. Regulatory: SEC.</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>payments, identity</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J28" s="3" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>Listed</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>Late-stage / major funding; B2B/infrastructure play (Payment Platform)</t>
         </is>
       </c>
-      <c r="N28" s="3" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="O28" s="3" t="inlineStr"/>
-      <c r="P28" s="3" t="inlineStr">
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
         <is>
           <t>בינונית</t>
         </is>
       </c>
-      <c r="Q28" s="3" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>https://www.zeepay.com</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>MNT Halan – DIGITALLY BANKING the unbanked</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Egypt</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
         <is>
           <t>https://www.mnt-halan.com</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>MNT Halan – DIGITALLY BANKING the unbanked In Egypt, MENA, and Africa Digitizing traditional banking and cash-based markets. +5 MN Total Clients Served MNT-Halan is Egypt’s Largest and Fastest Growing non-bank lender to the unbanked. 5 BN TOTAL LOANS DISBURSED Simple, Safe, and Efficient Digital payment solutions; mobile wallets and cards. Focus areas: payments, digital payments, mobile wallet, e-wallet, POS. Regulatory: SEC.</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>payments, digital payments, mobile wallet, e-wallet, POS, lending, digital lending, credit, loans, microfinance</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>Investment, Investors</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform)</t>
         </is>
       </c>
-      <c r="N29" s="3" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr"/>
-      <c r="P29" s="3" t="inlineStr">
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q29" s="3" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>https://www.mnt-halan.com</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Hubtel</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>dashboard to get real-time visibility</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>https://www.hubtel.com</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr"/>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
         <is>
           <t>Find and pay for everyday essentials and more with Hubtel Find and pay for everyday essentials from local retailers, food vendors and service providers Change Login Food Send Money Internet Data Utility Bills Airtime Car Insurance SMS Bet Topup Food Everyday Essentials Everyday Essentials Find whatever you want Order food, groceries and medicine, pay bills, send money
                   and more - all in one app Fast delivery in minutes Most orders arrive under 60 minutes. Track your order in
                   real time, every step of the way Choose, pay and receive Pay with card or mobile m...</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>payments, mobile money, mobile wallet, POS, API, insurance</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>Payment Platform</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>בינוני</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>Diverse product offering; B2B/infrastructure play (Payment Platform)</t>
         </is>
       </c>
-      <c r="N30" s="3" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr"/>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q30" s="3" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>https://www.hubtel.com</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>palmpay.com</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PalmPay</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
         <is>
           <t>https://www.palmpay.com</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
         <is>
           <t>No detailed information available from public sources.</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
         <is>
           <t>Fintech (General)</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="M31" s="4" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>Limited public information</t>
         </is>
       </c>
-      <c r="N31" s="4" t="inlineStr"/>
-      <c r="O31" s="4" t="inlineStr"/>
-      <c r="P31" s="4" t="inlineStr">
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
         <is>
           <t>נמוכה</t>
         </is>
       </c>
-      <c r="Q31" s="4" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>https://www.palmpay.com</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>FairMoney - Own Your Financial Journey</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr"/>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
         <is>
           <t>https://www.fairmoney.ng</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
         <is>
           <t>FairMoney - Own Your Financial Journey.</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
         <is>
           <t>Fintech (General)</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="M32" s="4" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>Limited public information</t>
         </is>
       </c>
-      <c r="N32" s="4" t="inlineStr"/>
-      <c r="O32" s="4" t="inlineStr"/>
-      <c r="P32" s="4" t="inlineStr">
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
         <is>
           <t>נמוכה</t>
         </is>
       </c>
-      <c r="Q32" s="4" t="inlineStr">
+      <c r="Q32" t="inlineStr">
         <is>
           <t>https://www.fairmoney.ng</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Nomba</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
         <is>
           <t>https://nomba.com</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
         <is>
           <t>No detailed information available from public sources.</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
         <is>
           <t>Fintech (General)</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr"/>
-      <c r="K33" s="4" t="inlineStr">
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="M33" s="4" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>Limited public information</t>
         </is>
       </c>
-      <c r="N33" s="4" t="inlineStr"/>
-      <c r="O33" s="4" t="inlineStr"/>
-      <c r="P33" s="4" t="inlineStr">
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
         <is>
           <t>נמוכה</t>
         </is>
       </c>
-      <c r="Q33" s="4" t="inlineStr">
+      <c r="Q33" t="inlineStr">
         <is>
           <t>https://nomba.com</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>TemboPlus</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr"/>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Tanzania</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
         <is>
           <t>https://temboplus.com</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>sales@temboplus.com</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
         <is>
           <t>TemboPlus Build &amp; Launch Financial Products Across Africa Infrastructure and Compliance to help companies build, launch and Scale Financial Services Across the continent. Products Product Portfolio: Engineered for Growth Seamlessly Integrate Banking and Payment Solutions I nfrastructure for Banking and Payments. Tembo provides secure, fully integrated APIs that enable neobanks, fintechs, and businesses to easily launch and scale financial services across Africa. Focus areas: payments, mobile money, neobank, cross-border, remittance. Regulatory: EMI, SEC.</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>payments, mobile money, neobank, cross-border, remittance, API, KYC, payroll</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Digital Bank / Neobank</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" s="4" t="inlineStr">
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="L34" s="4" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="M34" s="4" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>Diverse product offering; Contact info available</t>
         </is>
       </c>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>EMI, SEC</t>
         </is>
       </c>
-      <c r="O34" s="4" t="inlineStr"/>
-      <c r="P34" s="4" t="inlineStr">
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
         <is>
           <t>גבוהה</t>
         </is>
       </c>
-      <c r="Q34" s="4" t="inlineStr">
+      <c r="Q34" t="inlineStr">
         <is>
           <t>https://temboplus.com</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>IremboGov</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Rwanda</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
         <is>
           <t>https://www.irembo.gov.rw</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
         <is>
           <t>No detailed information available from public sources.</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
         <is>
           <t>Fintech (General)</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr"/>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="M35" s="4" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>Limited public information</t>
         </is>
       </c>
-      <c r="N35" s="4" t="inlineStr"/>
-      <c r="O35" s="4" t="inlineStr"/>
-      <c r="P35" s="4" t="inlineStr">
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
         <is>
           <t>נמוכה</t>
         </is>
       </c>
-      <c r="Q35" s="4" t="inlineStr">
+      <c r="Q35" t="inlineStr">
         <is>
           <t>https://www.irembo.gov.rw</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Santimpay</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr"/>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
         <is>
           <t>https://www.santimpay.com</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr"/>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
         <is>
           <t>No detailed information available from public sources.</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
         <is>
           <t>Fintech (General)</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr"/>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="L36" s="4" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>Limited public information</t>
         </is>
       </c>
-      <c r="N36" s="4" t="inlineStr"/>
-      <c r="O36" s="4" t="inlineStr"/>
-      <c r="P36" s="4" t="inlineStr">
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
         <is>
           <t>נמוכה</t>
         </is>
       </c>
-      <c r="Q36" s="4" t="inlineStr">
+      <c r="Q36" t="inlineStr">
         <is>
           <t>https://www.santimpay.com</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>AMOLE.NET - For Sale</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Amole</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Ethiopia</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
         <is>
           <t>https://www.amole.net</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
         <is>
           <t>+1 781-281-9475</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>02 Powered by Secure Exchange Prioritizing security above all else, we have forged a partnership with a globally renowned payment
 						processor and developed a state-of-the-art process for seamless transfers. Regulatory: SEC.</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
         <is>
           <t>Fintech (General)</t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>נמוך</t>
         </is>
       </c>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>Limited public information</t>
         </is>
       </c>
-      <c r="N37" s="4" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>SEC</t>
         </is>
       </c>
-      <c r="O37" s="4" t="inlineStr"/>
-      <c r="P37" s="4" t="inlineStr">
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
         <is>
           <t>נמוכה</t>
         </is>
       </c>
-      <c r="Q37" s="4" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>https://www.amole.net</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Rank</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Company Name</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Estimated Business Value</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Strategic Potential</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Key Reasons for Rating</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Flutterwave</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://flutterwave.com</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Diverse product offering; Late-stage / major funding; Pan-African presence (10 markets); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Major partnerships</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Moniepoint Inc.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://moniepoint.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Regulated / licensed; Diverse product offering; Late-stage / major funding; B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>FairMoney</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.getcarbon.co</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Regulated / licensed; Diverse product offering; Growth-stage funding; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence; Contact info available</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Mono</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://mono.co</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Diverse product offering; Growth-stage funding; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kora (KoraHQ)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.korahq.com</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Regulated / licensed; Diverse product offering; Growth-stage funding; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Major partnerships</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Stitch</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://stitch.money</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Regulated / licensed; Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Peach Payments</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://www.peachpayments.com</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Regulated / licensed; Diverse product offering; Multi-market (3 countries); B2B/infrastructure play (Payment Platform); Professional web presence; Contact info available; Major partnerships</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Ozow</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://www.ozow.com</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Regulated / licensed; Diverse product offering; B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence; Contact info available; Major partnerships</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Weaverfintech</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://www.weaverfintech.com</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Professional web presence; Major partnerships</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Adumo</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>https://www.adumo.com</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Diverse product offering; Growth-stage funding; B2B/infrastructure play (Payment Platform); Scale indicators (millions); Professional web presence; Contact info available; Major partnerships</t>
         </is>
       </c>
     </row>

</xml_diff>